<commit_message>
Added Po Amendment Test Scenarios & Fixed Failed Test Scenarios of HRM, PMF & POM
Added Po Amendment Test Scenarios & Fixed Failed Test Scenarios of HRM, PMF & POM
</commit_message>
<xml_diff>
--- a/testdata/LeaveAdjustmentData.xlsx
+++ b/testdata/LeaveAdjustmentData.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20490" windowHeight="7620"/>
+    <workbookView windowWidth="19200" windowHeight="6200"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1224,7 +1224,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="4"/>
+  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelRow="1" outlineLevelCol="4"/>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
@@ -1254,10 +1254,10 @@
         <v>1</v>
       </c>
       <c r="D2" s="3">
-        <v>45776</v>
+        <v>45990</v>
       </c>
       <c r="E2" s="3">
-        <v>45776</v>
+        <v>45990</v>
       </c>
     </row>
   </sheetData>

</xml_diff>